<commit_message>
Refresh S01, C01 and M01 outputs after end-to-end run; add first M01 Agent 3 to 5 results
</commit_message>
<xml_diff>
--- a/out/C01_chronic_care_patient_journey/agent5/agent5_qc_report.xlsx
+++ b/out/C01_chronic_care_patient_journey/agent5/agent5_qc_report.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every test judged" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Every test judged'!$A$1:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Every test judged'!$A$1:$I$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1031,7 +1031,7 @@
         <v>70</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
@@ -1111,7 +1111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1399,37 +1399,37 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
+          <t>HARNESS_FAULT</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>TC-FT15</t>
+          <t>TC-FT120</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Respondent Bot (not built yet)</t>
+          <t>Respondent Bot</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
+          <t>The bot could not carry the test out, so nothing was proved either way. This says nothing about the survey.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
+          <t>the journey never reached the point it was testing, so nothing about the survey was observed</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>fix the bot, then run this test again. Until then it is neither a pass nor a failure</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>TC-FT20</t>
+          <t>TC-FT15</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>TC-FT32</t>
+          <t>TC-FT20</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>TC-FT37</t>
+          <t>TC-FT32</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1552,12 +1552,12 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>TC-FT55</t>
+          <t>TC-FT37</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>TC-FT90</t>
+          <t>TC-FT55</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1626,12 +1626,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>TC-FT108</t>
+          <t>TC-FT90</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1663,12 +1663,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>TC-FT122, TC-FT123, TC-FT124, TC-FT125, TC-FT126</t>
+          <t>TC-FT108</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1700,12 +1700,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>TC-FT129, TC-FT130, TC-FT131, TC-FT132, TC-FT133</t>
+          <t>TC-FT122, TC-FT123, TC-FT124, TC-FT125, TC-FT126</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1732,37 +1732,37 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>NEEDS_SAMPLE</t>
+          <t>COVERAGE_GAP</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>TC-ST01</t>
+          <t>TC-FT129, TC-FT130, TC-FT131, TC-FT132, TC-FT133</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>nobody yet (needs a run with many respondents)</t>
+          <t>Respondent Bot (not built yet)</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
+          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
+          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
@@ -1774,12 +1774,12 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>TC-ST02</t>
+          <t>TC-ST01</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1811,12 +1811,12 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>TC-ST03</t>
+          <t>TC-ST02</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1848,12 +1848,12 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>TC-ST04</t>
+          <t>TC-ST03</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1885,30 +1885,67 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
+          <t>Q16</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>TC-ST04</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>nobody yet (needs a run with many respondents)</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>NEEDS_SAMPLE</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
           <t>Q19</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>TC-ST05</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>nobody yet (needs a run with many respondents)</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
@@ -1928,7 +1965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2773,11 +2810,11 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>TC-FT122</t>
+          <t>TC-FT120</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -2792,33 +2829,37 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O1 (North) admits a respondent while below target</t>
+          <t>answering D1 normally moves the respondent on to the question that should come next</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr"/>
+          <t>HARNESS_FAULT</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>D1 never appeared. The respondent was shown: S1, S2, S3, S4, Q1, Q2, Q3, Q4, Q5, Q6, Q7, Q8, Q9, Q10, Q11; D2 never appeared. The respondent was shown: S1, S2, S3, S4, Q1, Q2, Q3, Q4, Q5, Q6, Q7, Q8, Q9, Q10, Q11</t>
+        </is>
+      </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>fix the bot, then run this test again. Until then it is neither a pass nor a failure</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>TC-FT123</t>
+          <t>TC-FT122</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -2828,12 +2869,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O2 (South) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O1 (North) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -2855,11 +2896,11 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>TC-FT124</t>
+          <t>TC-FT123</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -2874,7 +2915,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O3 (East) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O2 (South) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -2896,11 +2937,11 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>TC-FT125</t>
+          <t>TC-FT124</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2915,7 +2956,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O4 (West) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O3 (East) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -2937,11 +2978,11 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>TC-FT126</t>
+          <t>TC-FT125</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2956,7 +2997,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O5 (Central) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O4 (West) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -2978,26 +3019,26 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>TC-FT129</t>
+          <t>TC-FT126</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O1 (21-29) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O5 (Central) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -3019,11 +3060,11 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>TC-FT130</t>
+          <t>TC-FT129</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -3033,12 +3074,12 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>P06</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O2 (30-39) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O1 (21-29) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -3060,11 +3101,11 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TC-FT131</t>
+          <t>TC-FT130</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -3079,7 +3120,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O3 (40-49) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O2 (30-39) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -3101,11 +3142,11 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>TC-FT132</t>
+          <t>TC-FT131</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -3120,7 +3161,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O4 (50-59) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O3 (40-49) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -3142,11 +3183,11 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>TC-FT133</t>
+          <t>TC-FT132</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -3161,7 +3202,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O5 (60+) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O4 (50-59) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -3181,8 +3222,49 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>142</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>TC-FT133</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>QUOTA_AGE:D2-O5 (60+) admits a respondent while below target</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>INCONCLUSIVE</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr"/>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I29"/>
+  <autoFilter ref="A1:I30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add display messages to S01, M01 and C01, supported from Agent 1 through the Respondent Bot
</commit_message>
<xml_diff>
--- a/out/C01_chronic_care_patient_journey/agent5/agent5_qc_report.xlsx
+++ b/out/C01_chronic_care_patient_journey/agent5/agent5_qc_report.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every test judged" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Every test judged'!$A$1:$I$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Every test judged'!$A$1:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -539,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -809,23 +809,23 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP, NEEDS_SAMPLE</t>
+          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP</t>
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Q16 presents all 6 items exactly once, with none missing and none repeated</t>
+          <t>QUOTA_REGION:D1-O2 (South) admits a respondent while below target</t>
         </is>
       </c>
     </row>
@@ -888,30 +888,30 @@
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>WORKING</t>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>BROKEN</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>every test on this journey passed</t>
+          <t>a respondent taking this journey would meet something wrong</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>reject rule R20 fires when its condition holds</t>
         </is>
       </c>
     </row>
@@ -938,14 +938,14 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>nothing on this journey is known to be wrong, but not everything could be proved: UNSETTLED_QUESTION, COVERAGE_GAP, NEEDS_SAMPLE</t>
+          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP, NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Q2 is not displayed when its guard fails</t>
+          <t>Q2's option list is narrowed to what was chosen at Q1</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Completing respondent — Q1=Independent provider; Q10=No; Q12=Not resolved</t>
+          <t>Completing respondent — Q5=None of these</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1017,30 +1017,30 @@
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>BROKEN</t>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>NOT PROVEN</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>a respondent taking this journey would meet something wrong</t>
+          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP, NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>70</v>
+        <v>6</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>56</v>
+        <v>4</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>reject rule R19 fires when its condition holds</t>
+          <t>Q16 presents all 6 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
     </row>
@@ -1052,43 +1052,86 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>Completing respondent — Q1=None of these; Q10=No; Q12=Not resolved</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>BROKEN</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>a respondent taking this journey would meet something wrong</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>reject rule R19 fires when its condition holds</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
           <t>Completing respondent — Q1=Care Network A; Q10=Yes; Q12=Fully</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>WORKING</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>every test on this journey passed</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="F16" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="G16" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="44" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="18" ht="44" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>WORKING means every test on this journey passed.
 BROKEN means a respondent taking it would meet something wrong: a defect in the survey, a misreading of the questionnaire, or a rule not built yet.
@@ -1098,7 +1141,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A18:I18"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1111,7 +1154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1187,7 +1230,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>TC-FT30</t>
+          <t>TC-FT33</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1224,7 +1267,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>TC-FT35</t>
+          <t>TC-FT40</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1261,7 +1304,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>TC-FT13</t>
+          <t>TC-FT14</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1298,7 +1341,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>TC-FT29</t>
+          <t>TC-FT32</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1330,12 +1373,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q17</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>TC-FT18</t>
+          <t>TC-FT102</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1350,7 +1393,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>this test depends on an unconfirmed reading: multi_equality, rule_precedence</t>
+          <t>this test depends on an unconfirmed reading: multi_equality, whitespace_is_an_answer</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1360,76 +1403,76 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>UNSETTLED_QUESTION</t>
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>TC-FT99</t>
+          <t>TC-FT16</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>the client</t>
+          <t>Respondent Bot (not built yet)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>The questionnaire never settled this, and a reading was assumed. Neither the survey nor the test is wrong until someone decides.</t>
+          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>this test depends on an unconfirmed reading: multi_equality, rule_precedence, whitespace_is_an_answer</t>
+          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>HARNESS_FAULT</t>
+          <t>COVERAGE_GAP</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>TC-FT120</t>
+          <t>TC-FT21</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Respondent Bot</t>
+          <t>Respondent Bot (not built yet)</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>The bot could not carry the test out, so nothing was proved either way. This says nothing about the survey.</t>
+          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>the journey never reached the point it was testing, so nothing about the survey was observed</t>
+          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>fix the bot, then run this test again. Until then it is neither a pass nor a failure</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1484,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>TC-FT15</t>
+          <t>TC-FT35</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1478,12 +1521,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>TC-FT20</t>
+          <t>TC-FT42</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1515,12 +1558,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>TC-FT32</t>
+          <t>TC-FT58</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1552,12 +1595,12 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>TC-FT37</t>
+          <t>TC-FT93</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1589,12 +1632,12 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>TC-FT55</t>
+          <t>TC-FT111</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1626,12 +1669,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>TC-FT90</t>
+          <t>TC-FT126, TC-FT127, TC-FT128, TC-FT129, TC-FT130</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1663,12 +1706,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>TC-FT108</t>
+          <t>TC-FT133, TC-FT134, TC-FT135, TC-FT136, TC-FT137</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1695,74 +1738,74 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
+          <t>NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>TC-FT122, TC-FT123, TC-FT124, TC-FT125, TC-FT126</t>
+          <t>TC-ST01</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Respondent Bot (not built yet)</t>
+          <t>nobody yet (needs a run with many respondents)</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
+          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
+          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
+          <t>NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>TC-FT129, TC-FT130, TC-FT131, TC-FT132, TC-FT133</t>
+          <t>TC-ST02</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Respondent Bot (not built yet)</t>
+          <t>nobody yet (needs a run with many respondents)</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
+          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
+          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
@@ -1774,12 +1817,12 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>TC-ST01</t>
+          <t>TC-ST03</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1811,12 +1854,12 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>TC-ST02</t>
+          <t>TC-ST04</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1848,12 +1891,12 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>TC-ST03</t>
+          <t>TC-ST05</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1872,80 +1915,6 @@
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Q16</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>TC-ST04</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>nobody yet (needs a run with many respondents)</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Q19</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>TC-ST05</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>nobody yet (needs a run with many respondents)</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
@@ -1965,7 +1934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2028,11 +1997,11 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>TC-FT13</t>
+          <t>TC-FT14</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -2042,7 +2011,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -2073,11 +2042,11 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>TC-FT15</t>
+          <t>TC-FT16</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -2087,7 +2056,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -2114,7 +2083,7 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -2128,7 +2097,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -2159,11 +2128,11 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>TC-FT18</t>
+          <t>TC-FT21</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -2178,78 +2147,78 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Q2 is not displayed when its guard fails</t>
+          <t>Q2's option list is narrowed to what was chosen at Q1</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>UNSETTLED_QUESTION</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Q2 appeared anyway, when it should have been hidden</t>
-        </is>
-      </c>
+          <t>INCONCLUSIVE</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>TC-FT20</t>
+          <t>TC-FT32</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Q2's option list is narrowed to what was chosen at Q1</t>
+          <t>Q5 rejects an answer breaking ['exclusive_option_id']</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr"/>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>TEST_MODEL_GAP</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
+        </is>
+      </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>check by hand that ticking the exclusive option clears the others. If it does, the rule works and the test should check the end state, not an error message</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>TC-FT29</t>
+          <t>TC-FT33</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -2259,12 +2228,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Q5 rejects an answer breaking ['exclusive_option_id']</t>
+          <t>reject rule R19 fires when its condition holds</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -2272,9 +2241,9 @@
           <t>FAILED</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>TEST_MODEL_GAP</t>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>NOT_BUILT_YET</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -2284,17 +2253,17 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>check by hand that ticking the exclusive option clears the others. If it does, the rule works and the test should check the end state, not an error message</t>
+          <t>no action on this test. It will pass once the survey builder emits that rule</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>TC-FT30</t>
+          <t>TC-FT35</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -2304,42 +2273,38 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>reject rule R19 fires when its condition holds</t>
+          <t>Q5 presents all 7 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>NOT_BUILT_YET</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It will pass once the survey builder emits that rule</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>TC-FT32</t>
+          <t>TC-ST02</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -2349,83 +2314,87 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Q5 presents all 7 items exactly once, with none missing and none repeated</t>
+          <t>Q5 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr"/>
+          <t>NEEDS_SAMPLE</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>needs several respondents, so it is not a single journey</t>
+        </is>
+      </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>TC-ST02</t>
+          <t>TC-FT40</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Q5 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>reject rule R20 fires when its condition holds</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>NEEDS_SAMPLE</t>
+          <t>NOT_BUILT_YET</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>needs several respondents, so it is not a single journey</t>
+          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+          <t>no action on this test. It will pass once the survey builder emits that rule</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>TC-FT35</t>
+          <t>TC-FT42</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2435,57 +2404,53 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>reject rule R20 fires when its condition holds</t>
+          <t>Q6's option list is narrowed to what was chosen at Q5</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>NOT_BUILT_YET</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It will pass once the survey builder emits that rule</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>TC-FT37</t>
+          <t>TC-FT58</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Q6's option list is narrowed to what was chosen at Q5</t>
+          <t>Q9 presents all 5 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -2507,11 +2472,11 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>TC-FT55</t>
+          <t>TC-ST03</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -2526,78 +2491,78 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Q9 presents all 5 items exactly once, with none missing and none repeated</t>
+          <t>Q9 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr"/>
+          <t>NEEDS_SAMPLE</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>needs several respondents, so it is not a single journey</t>
+        </is>
+      </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>TC-ST03</t>
+          <t>TC-FT93</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Q9 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>Q16 presents all 6 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>needs several respondents, so it is not a single journey</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>TC-FT90</t>
+          <t>TC-ST04</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -2607,128 +2572,128 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Q16 presents all 6 items exactly once, with none missing and none repeated</t>
+          <t>Q16 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr"/>
+          <t>NEEDS_SAMPLE</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>needs several respondents, so it is not a single journey</t>
+        </is>
+      </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>TC-ST04</t>
+          <t>TC-FT102</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>Q17</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P09</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Q16 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>Q17 refuses an answer of spaces alone, being compulsory</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>NEEDS_SAMPLE</t>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>UNSETTLED_QUESTION</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>needs several respondents, so it is not a single journey</t>
+          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>TC-FT99</t>
+          <t>TC-FT111</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Q17 refuses an answer of spaces alone, being compulsory</t>
+          <t>Q19 presents all 3 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>UNSETTLED_QUESTION</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
-        </is>
-      </c>
+          <t>INCONCLUSIVE</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>TC-FT108</t>
+          <t>TC-ST05</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -2738,83 +2703,83 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Q19 presents all 3 items exactly once, with none missing and none repeated</t>
+          <t>Q19 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr"/>
+          <t>NEEDS_SAMPLE</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>needs several respondents, so it is not a single journey</t>
+        </is>
+      </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>TC-ST05</t>
+          <t>TC-FT126</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Q19 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>QUOTA_REGION:D1-O1 (North) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>needs several respondents, so it is not a single journey</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>TC-FT120</t>
+          <t>TC-FT127</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -2824,42 +2789,38 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>answering D1 normally moves the respondent on to the question that should come next</t>
+          <t>QUOTA_REGION:D1-O2 (South) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>HARNESS_FAULT</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>D1 never appeared. The respondent was shown: S1, S2, S3, S4, Q1, Q2, Q3, Q4, Q5, Q6, Q7, Q8, Q9, Q10, Q11; D2 never appeared. The respondent was shown: S1, S2, S3, S4, Q1, Q2, Q3, Q4, Q5, Q6, Q7, Q8, Q9, Q10, Q11</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>fix the bot, then run this test again. Until then it is neither a pass nor a failure</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>TC-FT122</t>
+          <t>TC-FT128</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -2869,12 +2830,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O1 (North) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O3 (East) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -2896,11 +2857,11 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>TC-FT123</t>
+          <t>TC-FT129</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -2915,7 +2876,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O2 (South) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O4 (West) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -2937,11 +2898,11 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>TC-FT124</t>
+          <t>TC-FT130</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2956,7 +2917,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O3 (East) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O5 (Central) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -2978,26 +2939,26 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>TC-FT125</t>
+          <t>TC-FT133</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O4 (West) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O1 (21-29) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -3019,26 +2980,26 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>TC-FT126</t>
+          <t>TC-FT134</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O5 (Central) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O2 (30-39) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -3060,11 +3021,11 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>TC-FT129</t>
+          <t>TC-FT135</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -3074,12 +3035,12 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O1 (21-29) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O3 (40-49) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -3101,11 +3062,11 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TC-FT130</t>
+          <t>TC-FT136</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -3120,7 +3081,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O2 (30-39) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O4 (50-59) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -3142,11 +3103,11 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>TC-FT131</t>
+          <t>TC-FT137</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -3161,7 +3122,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O3 (40-49) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O5 (60+) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -3181,90 +3142,8 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
-        <v>141</v>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>TC-FT132</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>QUOTA_AGE:D2-O4 (50-59) admits a respondent while below target</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>INCONCLUSIVE</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
-        <v>142</v>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>TC-FT133</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>QUOTA_AGE:D2-O5 (60+) admits a respondent while below target</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>INCONCLUSIVE</t>
-        </is>
-      </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I30"/>
+  <autoFilter ref="A1:I28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
C01 Agent 5 report
</commit_message>
<xml_diff>
--- a/out/C01_chronic_care_patient_journey/agent5/agent5_qc_report.xlsx
+++ b/out/C01_chronic_care_patient_journey/agent5/agent5_qc_report.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every test judged" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Every test judged'!$A$1:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Every test judged'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -888,14 +888,14 @@
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>BROKEN</t>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>NOT PROVEN</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>a respondent taking this journey would meet something wrong</t>
+          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP, UNSETTLED_QUESTION</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
@@ -911,7 +911,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>reject rule R20 fires when its condition holds</t>
+          <t>Q6's option list is narrowed to what was chosen at Q5</t>
         </is>
       </c>
     </row>
@@ -938,14 +938,14 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP, NEEDS_SAMPLE</t>
+          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP, UNSETTLED_QUESTION, NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
         <v>30</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
@@ -974,30 +974,30 @@
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>NOT PROVEN</t>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>WORKING</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>nothing on this journey is known to be wrong, but not everything could be proved: UNSETTLED_QUESTION</t>
+          <t>every test on this journey passed</t>
         </is>
       </c>
       <c r="F13" s="4" t="n">
         <v>9</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Q17 refuses an answer of spaces alone, being compulsory</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1071,19 +1071,19 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q20</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>reject rule R19 fires when its condition holds</t>
+          <t>Q20's wording renders the answer given at Q19</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1225,12 +1225,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q20</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>TC-FT33</t>
+          <t>TC-FT114</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>before the run, Agent 3 already reported REJECT_RULE_NOT_BUILT for R19</t>
+          <t>before the run, Agent 3 already reported TEXT_PIPE_NOT_BUILT for Q20</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -1255,150 +1255,150 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>NOT_BUILT_YET</t>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>UNSETTLED_QUESTION</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>TC-FT40</t>
+          <t>TC-FT22</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Survey Builder (already on the backlog)</t>
+          <t>the client</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>The questionnaire asks for something the survey builder does not emit yet. Expected to fail until it does.</t>
+          <t>The questionnaire never settled this, and a reading was assumed. Neither the survey nor the test is wrong until someone decides.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>before the run, Agent 3 already reported REJECT_RULE_NOT_BUILT for R20</t>
+          <t>this test depends on an unconfirmed reading: multi_equality</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It will pass once the survey builder emits that rule</t>
+          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>TEST_MODEL_GAP</t>
+          <t>UNSETTLED_QUESTION</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>TC-FT43</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>the client</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>The questionnaire never settled this, and a reading was assumed. Neither the survey nor the test is wrong until someone decides.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>this test depends on an unconfirmed reading: multi_equality</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>TC-FT14</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Test Designer</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>The rule is enforced, but by a different mechanism than the test looks for. Nothing is broken; the test needs to learn the other way.</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>the survey was built with LimeSurvey's exclusive option (exclude_all_others), which unticks the other choices when the exclusive one is ticked. The respondent cannot submit both, so there is no error to show</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>check by hand that ticking the exclusive option clears the others. If it does, the rule works and the test should check the end state, not an error message</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>TEST_MODEL_GAP</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Q5</t>
-        </is>
-      </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>TC-FT32</t>
+          <t>TC-FT16</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Test Designer</t>
+          <t>Respondent Bot (not built yet)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>The rule is enforced, but by a different mechanism than the test looks for. Nothing is broken; the test needs to learn the other way.</t>
+          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>the survey was built with LimeSurvey's exclusive option (exclude_all_others), which unticks the other choices when the exclusive one is ticked. The respondent cannot submit both, so there is no error to show</t>
+          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>check by hand that ticking the exclusive option clears the others. If it does, the rule works and the test should check the end state, not an error message</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>UNSETTLED_QUESTION</t>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>TC-FT102</t>
+          <t>TC-FT21</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>the client</t>
+          <t>Respondent Bot (not built yet)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>The questionnaire never settled this, and a reading was assumed. Neither the survey nor the test is wrong until someone decides.</t>
+          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>this test depends on an unconfirmed reading: multi_equality, whitespace_is_an_answer</t>
+          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
@@ -1410,12 +1410,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>TC-FT16</t>
+          <t>TC-FT35</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1447,12 +1447,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>TC-FT21</t>
+          <t>TC-FT42</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>TC-FT35</t>
+          <t>TC-FT58</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1521,12 +1521,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>TC-FT42</t>
+          <t>TC-FT93</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1558,12 +1558,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>TC-FT58</t>
+          <t>TC-FT111</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1595,12 +1595,12 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>TC-FT93</t>
+          <t>TC-FT125, TC-FT126, TC-FT127, TC-FT128, TC-FT129</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1632,12 +1632,12 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>TC-FT111</t>
+          <t>TC-FT132, TC-FT133, TC-FT134, TC-FT135, TC-FT136</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1664,74 +1664,74 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
+          <t>NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>TC-FT126, TC-FT127, TC-FT128, TC-FT129, TC-FT130</t>
+          <t>TC-ST01</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Respondent Bot (not built yet)</t>
+          <t>nobody yet (needs a run with many respondents)</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
+          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
+          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
+          <t>NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>TC-FT133, TC-FT134, TC-FT135, TC-FT136, TC-FT137</t>
+          <t>TC-ST02</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Respondent Bot (not built yet)</t>
+          <t>nobody yet (needs a run with many respondents)</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
+          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
+          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
@@ -1743,12 +1743,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>TC-ST01</t>
+          <t>TC-ST03</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1780,12 +1780,12 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>TC-ST02</t>
+          <t>TC-ST04</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1817,12 +1817,12 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>TC-ST03</t>
+          <t>TC-ST05</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1841,80 +1841,6 @@
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Q16</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>TC-ST04</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>nobody yet (needs a run with many respondents)</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Q19</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>TC-ST05</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>nobody yet (needs a run with many respondents)</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
@@ -1934,7 +1860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1997,11 +1923,11 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>TC-FT14</t>
+          <t>TC-FT16</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -2016,37 +1942,33 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Q1 rejects an answer breaking ['exclusive_option_id']</t>
+          <t>Q1 presents all 5 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="G2" s="10" t="inlineStr">
-        <is>
-          <t>TEST_MODEL_GAP</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
-        </is>
-      </c>
+          <t>INCONCLUSIVE</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr"/>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>check by hand that ticking the exclusive option clears the others. If it does, the rule works and the test should check the end state, not an error message</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>TC-FT16</t>
+          <t>TC-ST01</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -2061,78 +1983,78 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Q1 presents all 5 items exactly once, with none missing and none repeated</t>
+          <t>Q1 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr"/>
+          <t>NEEDS_SAMPLE</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>needs several respondents, so it is not a single journey</t>
+        </is>
+      </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>TC-ST01</t>
+          <t>TC-FT21</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Q1 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>Q2's option list is narrowed to what was chosen at Q1</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>needs several respondents, so it is not a single journey</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>TC-FT21</t>
+          <t>TC-FT22</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -2147,33 +2069,37 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Q2's option list is narrowed to what was chosen at Q1</t>
+          <t>Q2 is shown by its guard and simultaneously reflects its dependency on Q1</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr"/>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>UNSETTLED_QUESTION</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>it did not. Q2 read: 'Which brands would you consider?'</t>
+        </is>
+      </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>TC-FT32</t>
+          <t>TC-FT35</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -2188,37 +2114,33 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Q5 rejects an answer breaking ['exclusive_option_id']</t>
+          <t>Q5 presents all 7 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>TEST_MODEL_GAP</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
-        </is>
-      </c>
+          <t>INCONCLUSIVE</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>check by hand that ticking the exclusive option clears the others. If it does, the rule works and the test should check the end state, not an error message</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>TC-FT33</t>
+          <t>TC-ST02</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -2233,52 +2155,52 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>reject rule R19 fires when its condition holds</t>
+          <t>Q5 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>NOT_BUILT_YET</t>
+          <t>NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
+          <t>needs several respondents, so it is not a single journey</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It will pass once the survey builder emits that rule</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>TC-FT35</t>
+          <t>TC-FT42</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Q5 presents all 7 items exactly once, with none missing and none repeated</t>
+          <t>Q6's option list is narrowed to what was chosen at Q5</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -2300,157 +2222,157 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>TC-ST02</t>
+          <t>TC-FT43</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Q5 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>Q6 is shown by its guard and simultaneously reflects its dependency on Q5</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>NEEDS_SAMPLE</t>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>UNSETTLED_QUESTION</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>needs several respondents, so it is not a single journey</t>
+          <t>it did not. Q6 read: 'Which touchpoint was most influential?'</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>TC-FT40</t>
+          <t>TC-FT58</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>reject rule R20 fires when its condition holds</t>
+          <t>Q9 presents all 5 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>NOT_BUILT_YET</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It will pass once the survey builder emits that rule</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>TC-FT42</t>
+          <t>TC-ST03</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Q6's option list is narrowed to what was chosen at Q5</t>
+          <t>Q9 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr"/>
+          <t>NEEDS_SAMPLE</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>needs several respondents, so it is not a single journey</t>
+        </is>
+      </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>TC-FT58</t>
+          <t>TC-FT93</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Q9 presents all 5 items exactly once, with none missing and none repeated</t>
+          <t>Q16 presents all 6 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -2472,26 +2394,26 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>65</v>
+        <v>101</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>TC-ST03</t>
+          <t>TC-ST04</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Q9 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>Q16 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -2517,26 +2439,26 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>TC-FT93</t>
+          <t>TC-FT111</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Q16 presents all 6 items exactly once, with none missing and none repeated</t>
+          <t>Q19 presents all 3 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -2558,26 +2480,26 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>TC-ST04</t>
+          <t>TC-ST05</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Q16 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>Q19 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -2603,26 +2525,26 @@
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>TC-FT102</t>
+          <t>TC-FT114</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q20</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>P09</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Q17 refuses an answer of spaces alone, being compulsory</t>
+          <t>Q20's wording renders the answer given at Q19</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -2630,34 +2552,34 @@
           <t>FAILED</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>UNSETTLED_QUESTION</t>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>NOT_BUILT_YET</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>it accepted the answer and moved on, when it should have stopped the respondent</t>
+          <t>it did not. Q20 read: 'How appealing is the selected proposition?'</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
+          <t>no action on this test. It will pass once the survey builder emits that rule</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>TC-FT111</t>
+          <t>TC-FT125</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -2667,7 +2589,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Q19 presents all 3 items exactly once, with none missing and none repeated</t>
+          <t>QUOTA_REGION:D1-O1 (North) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -2689,56 +2611,52 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>TC-ST05</t>
+          <t>TC-FT126</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Q19 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>QUOTA_REGION:D1-O2 (South) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>needs several respondents, so it is not a single journey</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>TC-FT126</t>
+          <t>TC-FT127</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2748,12 +2666,12 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O1 (North) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O3 (East) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -2775,11 +2693,11 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>TC-FT127</t>
+          <t>TC-FT128</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -2794,7 +2712,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O2 (South) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O4 (West) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -2816,11 +2734,11 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>TC-FT128</t>
+          <t>TC-FT129</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -2835,7 +2753,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O3 (East) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O5 (Central) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -2857,26 +2775,26 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>TC-FT129</t>
+          <t>TC-FT132</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O4 (West) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O1 (21-29) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -2898,26 +2816,26 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>TC-FT130</t>
+          <t>TC-FT133</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O5 (Central) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O2 (30-39) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -2939,11 +2857,11 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>TC-FT133</t>
+          <t>TC-FT134</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2953,12 +2871,12 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O1 (21-29) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O3 (40-49) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -2980,11 +2898,11 @@
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>TC-FT134</t>
+          <t>TC-FT135</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -2999,7 +2917,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O2 (30-39) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O4 (50-59) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -3021,11 +2939,11 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>TC-FT135</t>
+          <t>TC-FT136</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -3040,7 +2958,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O3 (40-49) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O5 (60+) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -3060,90 +2978,8 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
-        <v>145</v>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>TC-FT136</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>QUOTA_AGE:D2-O4 (50-59) admits a respondent while below target</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>INCONCLUSIVE</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
-        <v>146</v>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>TC-FT137</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>QUOTA_AGE:D2-O5 (60+) admits a respondent while below target</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>INCONCLUSIVE</t>
-        </is>
-      </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I28"/>
+  <autoFilter ref="A1:I26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bot and Agent 5 runs: S01, M01, C01 on the current build
</commit_message>
<xml_diff>
--- a/out/C01_chronic_care_patient_journey/agent5/agent5_qc_report.xlsx
+++ b/out/C01_chronic_care_patient_journey/agent5/agent5_qc_report.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Every test judged" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Every test judged'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Every test judged'!$A$1:$I$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,14 +75,8 @@
       <color rgb="00635E7E"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="004338A8"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -114,11 +108,6 @@
         <fgColor rgb="00EFEFEF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E4E1F7"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -146,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -169,9 +158,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -895,14 +881,14 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP, UNSETTLED_QUESTION</t>
+          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
         <v>23</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -938,14 +924,14 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP, UNSETTLED_QUESTION, NEEDS_SAMPLE</t>
+          <t>nothing on this journey is known to be wrong, but not everything could be proved: COVERAGE_GAP, NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="F12" s="4" t="n">
         <v>30</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
@@ -1154,7 +1140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1255,76 +1241,76 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>UNSETTLED_QUESTION</t>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>TC-FT16</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Respondent Bot (not built yet)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>TC-FT22</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>the client</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>The questionnaire never settled this, and a reading was assumed. Neither the survey nor the test is wrong until someone decides.</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>this test depends on an unconfirmed reading: multi_equality</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>UNSETTLED_QUESTION</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>TC-FT43</t>
+          <t>TC-FT21</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>the client</t>
+          <t>Respondent Bot (not built yet)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>The questionnaire never settled this, and a reading was assumed. Neither the survey nor the test is wrong until someone decides.</t>
+          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>this test depends on an unconfirmed reading: multi_equality</t>
+          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
@@ -1336,12 +1322,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>TC-FT16</t>
+          <t>TC-FT35</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1373,12 +1359,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>TC-FT21</t>
+          <t>TC-FT42</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1410,12 +1396,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>TC-FT35</t>
+          <t>TC-FT58</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1447,12 +1433,12 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>TC-FT42</t>
+          <t>TC-FT93</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1484,12 +1470,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>TC-FT58</t>
+          <t>TC-FT111</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1521,12 +1507,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>TC-FT93</t>
+          <t>TC-FT125, TC-FT126, TC-FT127, TC-FT128, TC-FT129</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1558,12 +1544,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>TC-FT111</t>
+          <t>TC-FT132, TC-FT133, TC-FT134, TC-FT135, TC-FT136</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1590,74 +1576,74 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
+          <t>NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>TC-FT125, TC-FT126, TC-FT127, TC-FT128, TC-FT129</t>
+          <t>TC-ST01</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Respondent Bot (not built yet)</t>
+          <t>nobody yet (needs a run with many respondents)</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
+          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
+          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
+          <t>NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>TC-FT132, TC-FT133, TC-FT134, TC-FT135, TC-FT136</t>
+          <t>TC-ST02</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Respondent Bot (not built yet)</t>
+          <t>nobody yet (needs a run with many respondents)</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>The bot reached the right place but does not yet know how to observe this kind of claim, so nothing was proved either way. Nothing is known to be wrong.</t>
+          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>the bot reached the right place but has no way yet to observe this kind of claim</t>
+          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
@@ -1669,12 +1655,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>TC-ST01</t>
+          <t>TC-ST03</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1706,12 +1692,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>TC-ST02</t>
+          <t>TC-ST04</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1743,12 +1729,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>TC-ST03</t>
+          <t>TC-ST05</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1767,80 +1753,6 @@
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Q16</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>TC-ST04</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>nobody yet (needs a run with many respondents)</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Q19</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>TC-ST05</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>nobody yet (needs a run with many respondents)</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>This can only be checked across many respondents, such as the order options are shown in. One run through the survey cannot prove it, so it was never going to run as a single journey.</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>the claim is about what happens across many respondents, so it is not a single journey and the bot rightly did not run it</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
@@ -1860,7 +1772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2050,56 +1962,52 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>TC-FT22</t>
+          <t>TC-FT35</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Q2 is shown by its guard and simultaneously reflects its dependency on Q1</t>
+          <t>Q5 presents all 7 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>UNSETTLED_QUESTION</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>it did not. Q2 read: 'Which brands would you consider?'</t>
-        </is>
-      </c>
+          <t>INCONCLUSIVE</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>TC-FT35</t>
+          <t>TC-ST02</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -2114,93 +2022,93 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Q5 presents all 7 items exactly once, with none missing and none repeated</t>
+          <t>Q5 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr"/>
+          <t>NEEDS_SAMPLE</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>needs several respondents, so it is not a single journey</t>
+        </is>
+      </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>TC-ST02</t>
+          <t>TC-FT42</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P07</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Q5 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>Q6's option list is narrowed to what was chosen at Q5</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>needs several respondents, so it is not a single journey</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>TC-FT42</t>
+          <t>TC-FT58</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Q6's option list is narrowed to what was chosen at Q5</t>
+          <t>Q9 presents all 5 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -2222,71 +2130,71 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>TC-FT43</t>
+          <t>TC-ST03</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q9</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>P07</t>
+          <t>P08</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Q6 is shown by its guard and simultaneously reflects its dependency on Q5</t>
+          <t>Q9 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>UNSETTLED_QUESTION</t>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>NEEDS_SAMPLE</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>it did not. Q6 read: 'Which touchpoint was most influential?'</t>
+          <t>needs several respondents, so it is not a single journey</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>ask the client which reading is intended. Until then this is a question, not a defect</t>
+          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>TC-FT58</t>
+          <t>TC-FT93</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Q9 presents all 5 items exactly once, with none missing and none repeated</t>
+          <t>Q16 presents all 6 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -2308,26 +2216,26 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>65</v>
+        <v>101</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>TC-ST03</t>
+          <t>TC-ST04</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q16</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>P08</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Q9 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>Q16 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -2353,26 +2261,26 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>TC-FT93</t>
+          <t>TC-FT111</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Q16 presents all 6 items exactly once, with none missing and none repeated</t>
+          <t>Q19 presents all 3 items exactly once, with none missing and none repeated</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -2394,26 +2302,26 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>TC-ST04</t>
+          <t>TC-ST05</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Q16</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Q16 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>Q19 presents its items in a different order to different respondents, proving shuffling is switched on</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -2439,16 +2347,16 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>TC-FT111</t>
+          <t>TC-FT114</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Q20</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -2458,38 +2366,42 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Q19 presents all 3 items exactly once, with none missing and none repeated</t>
+          <t>Q20's wording renders the answer given at Q19</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>INCONCLUSIVE</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr"/>
+          <t>NOT_BUILT_YET</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>it did not. Q20 read: 'How appealing is the selected proposition? Choose one of the following answers Very poor P'</t>
+        </is>
+      </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
+          <t>no action on this test. It will pass once the survey builder emits that rule</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>TC-ST05</t>
+          <t>TC-FT125</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -2499,82 +2411,74 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Q19 presents its items in a different order to different respondents, proving shuffling is switched on</t>
+          <t>QUOTA_REGION:D1-O1 (North) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>SKIPPED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>NEEDS_SAMPLE</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>needs several respondents, so it is not a single journey</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It needs a run with a sample, which does not exist yet</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>TC-FT114</t>
+          <t>TC-FT126</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Q20</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Q20's wording renders the answer given at Q19</t>
+          <t>QUOTA_REGION:D1-O2 (South) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>INCONCLUSIVE</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>NOT_BUILT_YET</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>it did not. Q20 read: 'How appealing is the selected proposition?'</t>
-        </is>
-      </c>
+          <t>COVERAGE_GAP</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>no action on this test. It will pass once the survey builder emits that rule</t>
+          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>TC-FT125</t>
+          <t>TC-FT127</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -2584,12 +2488,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P05</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O1 (North) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O3 (East) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -2611,11 +2515,11 @@
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>TC-FT126</t>
+          <t>TC-FT128</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -2630,7 +2534,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O2 (South) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O4 (West) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -2652,11 +2556,11 @@
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>TC-FT127</t>
+          <t>TC-FT129</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2671,7 +2575,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O3 (East) admits a respondent while below target</t>
+          <t>QUOTA_REGION:D1-O5 (Central) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -2693,26 +2597,26 @@
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>TC-FT128</t>
+          <t>TC-FT132</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O4 (West) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O1 (21-29) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -2734,26 +2638,26 @@
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>TC-FT129</t>
+          <t>TC-FT133</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>P05</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_REGION:D1-O5 (Central) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O2 (30-39) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -2775,11 +2679,11 @@
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>TC-FT132</t>
+          <t>TC-FT134</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -2789,12 +2693,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>P11</t>
+          <t>P06</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O1 (21-29) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O3 (40-49) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -2816,11 +2720,11 @@
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>TC-FT133</t>
+          <t>TC-FT135</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -2835,7 +2739,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O2 (30-39) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O4 (50-59) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -2857,11 +2761,11 @@
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>TC-FT134</t>
+          <t>TC-FT136</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -2876,7 +2780,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>QUOTA_AGE:D2-O3 (40-49) admits a respondent while below target</t>
+          <t>QUOTA_AGE:D2-O5 (60+) admits a respondent while below target</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -2896,90 +2800,8 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
-        <v>144</v>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>TC-FT135</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>QUOTA_AGE:D2-O4 (50-59) admits a respondent while below target</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>INCONCLUSIVE</t>
-        </is>
-      </c>
-      <c r="G25" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
-        <v>145</v>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>TC-FT136</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>QUOTA_AGE:D2-O5 (60+) admits a respondent while below target</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>INCONCLUSIVE</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>teach the bot to observe it, or record that this claim cannot be proved by running one respondent through the survey</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I26"/>
+  <autoFilter ref="A1:I24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>